<commit_message>
Agrega 4 procedimientos faltantes y enlaza políticas↔procedimientos en ambos sentidos
- Nuevos procedimientos (.docx, formato del set): PROC-SGSI-15 Desarrollo seguro
  (SDLC, cierra G-13), 16 Respuesta ante malware (POL-04), 17 Uso seguro de
  dispositivos (POL-06), 18 Cifrado y gestión de llaves (POL-12).
- Hipervínculos clicables en ambos sentidos: cada política enlaza su(s)
  procedimiento(s) y cada procedimiento su política base (Ctrl+clic en Word/LO).
  Las 15 políticas quedan con procedimiento dedicado (POL-04/06/12 → 16/17/18;
  PROC-15 SDLC referenciado desde POL-09 y POL-15).
- Índices: Maestro (54 docs, 18 procedimientos), mapeo ISO, READMEs,
  Gap Analysis (G-13/G-14 resueltos) y RACI (proceso 20 SDLC → PROC-15).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Maestro Documental SGSI.xlsx
+++ b/docs/Maestro Documental SGSI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Maestro Documental" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maestro Documental" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Maestro Documental'!$A$3:$L$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Maestro Documental'!$A$3:$L$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="12" min="1" max="1"/>
@@ -2942,17 +2942,17 @@
     <row r="42" ht="28" customHeight="1" s="13">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>ANR-SGSI-01</t>
+          <t>PROC-SGSI-15</t>
         </is>
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>Metodología de Evaluación y Tratamiento de Riesgos</t>
+          <t>Procedimiento de desarrollo seguro (SDLC)</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>Análisis de riesgos</t>
+          <t>Procedimiento</t>
         </is>
       </c>
       <c r="D42" s="19" t="inlineStr">
@@ -2972,12 +2972,12 @@
       </c>
       <c r="G42" s="18" t="inlineStr">
         <is>
-          <t>CISO</t>
+          <t>Jefe de Desarrollo / CISO</t>
         </is>
       </c>
       <c r="H42" s="18" t="inlineStr">
         <is>
-          <t>Comité SGSI</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="I42" s="20" t="inlineStr">
@@ -2992,29 +2992,29 @@
       </c>
       <c r="K42" s="18" t="inlineStr">
         <is>
-          <t>Cl. 6.1.2</t>
+          <t>8.4, 8.25, 8.26, 8.27, 8.28, 8.29, 8.31</t>
         </is>
       </c>
       <c r="L42" s="18" t="inlineStr">
         <is>
-          <t>ISO 27001; NIST CSF GV.RM/ID.RA</t>
+          <t>PCI DSS Req 6</t>
         </is>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1" s="13">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>ANR-SGSI-02</t>
+          <t>PROC-SGSI-16</t>
         </is>
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>Plan de Tratamiento de Riesgos</t>
+          <t>Procedimiento de respuesta ante malware</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Análisis de riesgos</t>
+          <t>Procedimiento</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3034,12 +3034,12 @@
       </c>
       <c r="G43" s="18" t="inlineStr">
         <is>
-          <t>CISO</t>
+          <t>Ciberseguridad / Gerencia TI</t>
         </is>
       </c>
       <c r="H43" s="18" t="inlineStr">
         <is>
-          <t>Comité SGSI</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="I43" s="20" t="inlineStr">
@@ -3054,29 +3054,29 @@
       </c>
       <c r="K43" s="18" t="inlineStr">
         <is>
-          <t>Cl. 6.1.3</t>
+          <t>8.7</t>
         </is>
       </c>
       <c r="L43" s="18" t="inlineStr">
         <is>
-          <t>ISO 27001; NIST CSF GV.RM</t>
+          <t>PCI DSS Req 5</t>
         </is>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1" s="13">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>ANR-SGSI-03</t>
+          <t>PROC-SGSI-17</t>
         </is>
       </c>
       <c r="B44" s="18" t="inlineStr">
         <is>
-          <t>Inventario de Activos de Información (15 activos)</t>
+          <t>Procedimiento de uso seguro de dispositivos</t>
         </is>
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Análisis de riesgos</t>
+          <t>Procedimiento</t>
         </is>
       </c>
       <c r="D44" s="19" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="G44" s="18" t="inlineStr">
         <is>
-          <t>CISO / Dueños de activos</t>
+          <t>Gerencia TI</t>
         </is>
       </c>
       <c r="H44" s="18" t="inlineStr">
@@ -3116,29 +3116,29 @@
       </c>
       <c r="K44" s="18" t="inlineStr">
         <is>
-          <t>A.5.9</t>
+          <t>8.1, 7.9, 6.7</t>
         </is>
       </c>
       <c r="L44" s="18" t="inlineStr">
         <is>
-          <t>NIST CSF ID.AM</t>
+          <t>PCI DSS Req 9</t>
         </is>
       </c>
     </row>
     <row r="45" ht="28" customHeight="1" s="13">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>ANR-SGSI-04</t>
+          <t>PROC-SGSI-18</t>
         </is>
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>Matriz de Evaluación de Riesgos (R-01 a R-17)</t>
+          <t>Procedimiento de cifrado y gestión de llaves</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Análisis de riesgos</t>
+          <t>Procedimiento</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3158,12 +3158,12 @@
       </c>
       <c r="G45" s="18" t="inlineStr">
         <is>
-          <t>CISO</t>
+          <t>Gerencia TI / DBA</t>
         </is>
       </c>
       <c r="H45" s="18" t="inlineStr">
         <is>
-          <t>Comité SGSI</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="I45" s="20" t="inlineStr">
@@ -3178,24 +3178,24 @@
       </c>
       <c r="K45" s="18" t="inlineStr">
         <is>
-          <t>Cl. 6.1.2</t>
+          <t>8.24</t>
         </is>
       </c>
       <c r="L45" s="18" t="inlineStr">
         <is>
-          <t>NIST CSF ID.RA</t>
+          <t>Ley 19.628; PCI DSS Req 3, 4</t>
         </is>
       </c>
     </row>
     <row r="46" ht="28" customHeight="1" s="13">
       <c r="A46" s="17" t="inlineStr">
         <is>
-          <t>ANR-SGSI-05</t>
+          <t>ANR-SGSI-01</t>
         </is>
       </c>
       <c r="B46" s="18" t="inlineStr">
         <is>
-          <t>Declaración de Aplicabilidad (SoA) — controles tecnológicos 8.1–8.34</t>
+          <t>Metodología de Evaluación y Tratamiento de Riesgos</t>
         </is>
       </c>
       <c r="C46" s="19" t="inlineStr">
@@ -3240,24 +3240,24 @@
       </c>
       <c r="K46" s="18" t="inlineStr">
         <is>
-          <t>Cl. 6.1.3.d</t>
+          <t>Cl. 6.1.2</t>
         </is>
       </c>
       <c r="L46" s="18" t="inlineStr">
         <is>
-          <t>ISO 27001 Anexo A (cap. 8)</t>
+          <t>ISO 27001; NIST CSF GV.RM/ID.RA</t>
         </is>
       </c>
     </row>
     <row r="47" ht="28" customHeight="1" s="13">
       <c r="A47" s="17" t="inlineStr">
         <is>
-          <t>ANR-SGSI-06</t>
+          <t>ANR-SGSI-02</t>
         </is>
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>Gap Analysis y Estado del SGSI</t>
+          <t>Plan de Tratamiento de Riesgos</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
@@ -3282,12 +3282,12 @@
       </c>
       <c r="G47" s="18" t="inlineStr">
         <is>
-          <t>Equipo SGSI</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>CISO</t>
+          <t>Comité SGSI</t>
         </is>
       </c>
       <c r="I47" s="20" t="inlineStr">
@@ -3302,29 +3302,29 @@
       </c>
       <c r="K47" s="18" t="inlineStr">
         <is>
-          <t>Cl. 4–10</t>
+          <t>Cl. 6.1.3</t>
         </is>
       </c>
       <c r="L47" s="18" t="inlineStr">
         <is>
-          <t>NIST CSF</t>
+          <t>ISO 27001; NIST CSF GV.RM</t>
         </is>
       </c>
     </row>
     <row r="48" ht="28" customHeight="1" s="13">
       <c r="A48" s="17" t="inlineStr">
         <is>
-          <t>DOC-SGSI-01</t>
+          <t>ANR-SGSI-03</t>
         </is>
       </c>
       <c r="B48" s="18" t="inlineStr">
         <is>
-          <t>Maestro Documental del SGSI</t>
+          <t>Inventario de Activos de Información (15 activos)</t>
         </is>
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Gestión documental</t>
+          <t>Análisis de riesgos</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="G48" s="18" t="inlineStr">
         <is>
-          <t>Equipo SGSI</t>
+          <t>CISO / Dueños de activos</t>
         </is>
       </c>
       <c r="H48" s="18" t="inlineStr">
@@ -3364,29 +3364,29 @@
       </c>
       <c r="K48" s="18" t="inlineStr">
         <is>
-          <t>Cl. 7.5</t>
+          <t>A.5.9</t>
         </is>
       </c>
       <c r="L48" s="18" t="inlineStr">
         <is>
-          <t>ISO 27001</t>
+          <t>NIST CSF ID.AM</t>
         </is>
       </c>
     </row>
     <row r="49" ht="28" customHeight="1" s="13">
       <c r="A49" s="17" t="inlineStr">
         <is>
-          <t>DOC-SGSI-02</t>
+          <t>ANR-SGSI-04</t>
         </is>
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>Matriz Legal</t>
+          <t>Matriz de Evaluación de Riesgos (R-01 a R-17)</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Gestión documental</t>
+          <t>Análisis de riesgos</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="G49" s="18" t="inlineStr">
         <is>
-          <t>CISO / Legal</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="H49" s="18" t="inlineStr">
@@ -3426,29 +3426,29 @@
       </c>
       <c r="K49" s="18" t="inlineStr">
         <is>
-          <t>Cl. 4.2</t>
+          <t>Cl. 6.1.2</t>
         </is>
       </c>
       <c r="L49" s="18" t="inlineStr">
         <is>
-          <t>Ley 21.663; Ley 19.628; PCI DSS v4.0</t>
+          <t>NIST CSF ID.RA</t>
         </is>
       </c>
     </row>
     <row r="50" ht="28" customHeight="1" s="13">
       <c r="A50" s="17" t="inlineStr">
         <is>
-          <t>DOC-SGSI-03</t>
+          <t>ANR-SGSI-05</t>
         </is>
       </c>
       <c r="B50" s="18" t="inlineStr">
         <is>
-          <t>Matriz de Competencias</t>
+          <t>Declaración de Aplicabilidad (SoA) — controles tecnológicos 8.1–8.34</t>
         </is>
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Gestión documental</t>
+          <t>Análisis de riesgos</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="G50" s="18" t="inlineStr">
         <is>
-          <t>RRHH / CISO</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="H50" s="18" t="inlineStr">
@@ -3488,29 +3488,29 @@
       </c>
       <c r="K50" s="18" t="inlineStr">
         <is>
-          <t>Cl. 7.2 · A.6.3</t>
+          <t>Cl. 6.1.3.d</t>
         </is>
       </c>
       <c r="L50" s="18" t="inlineStr">
         <is>
-          <t>ISO 27001</t>
+          <t>ISO 27001 Anexo A (cap. 8)</t>
         </is>
       </c>
     </row>
     <row r="51" ht="28" customHeight="1" s="13">
       <c r="A51" s="17" t="inlineStr">
         <is>
-          <t>DOC-SGSI-04</t>
+          <t>ANR-SGSI-06</t>
         </is>
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>Mapeo SGSI ↔ ISO 27001:2022 (Anexo A)</t>
+          <t>Gap Analysis y Estado del SGSI</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Gestión documental</t>
+          <t>Análisis de riesgos</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="G51" s="18" t="inlineStr">
         <is>
-          <t>CISO</t>
+          <t>Equipo SGSI</t>
         </is>
       </c>
       <c r="H51" s="18" t="inlineStr">
@@ -3550,24 +3550,24 @@
       </c>
       <c r="K51" s="18" t="inlineStr">
         <is>
-          <t>Anexo A</t>
+          <t>Cl. 4–10</t>
         </is>
       </c>
       <c r="L51" s="18" t="inlineStr">
         <is>
-          <t>ISO 27001</t>
+          <t>NIST CSF</t>
         </is>
       </c>
     </row>
     <row r="52" ht="28" customHeight="1" s="13">
       <c r="A52" s="17" t="inlineStr">
         <is>
-          <t>DOC-SGSI-05</t>
+          <t>DOC-SGSI-01</t>
         </is>
       </c>
       <c r="B52" s="18" t="inlineStr">
         <is>
-          <t>Contrato de Trabajo y Anexo de Seguridad</t>
+          <t>Maestro Documental del SGSI</t>
         </is>
       </c>
       <c r="C52" s="19" t="inlineStr">
@@ -3592,12 +3592,12 @@
       </c>
       <c r="G52" s="18" t="inlineStr">
         <is>
-          <t>RRHH</t>
+          <t>Equipo SGSI</t>
         </is>
       </c>
       <c r="H52" s="18" t="inlineStr">
         <is>
-          <t>Gerencia General</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="I52" s="20" t="inlineStr">
@@ -3607,105 +3607,353 @@
       </c>
       <c r="J52" s="19" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Interno</t>
         </is>
       </c>
       <c r="K52" s="18" t="inlineStr">
         <is>
-          <t>A.6.1, A.6.2, A.6.6</t>
+          <t>Cl. 7.5</t>
         </is>
       </c>
       <c r="L52" s="18" t="inlineStr">
         <is>
-          <t>Ley 19.628; ISO Personas (6)</t>
+          <t>ISO 27001</t>
         </is>
       </c>
     </row>
     <row r="53" ht="28" customHeight="1" s="13">
       <c r="A53" s="17" t="inlineStr">
         <is>
+          <t>DOC-SGSI-02</t>
+        </is>
+      </c>
+      <c r="B53" s="18" t="inlineStr">
+        <is>
+          <t>Matriz Legal</t>
+        </is>
+      </c>
+      <c r="C53" s="19" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E53" s="19" t="inlineStr">
+        <is>
+          <t>17-06-2026</t>
+        </is>
+      </c>
+      <c r="F53" s="19" t="inlineStr">
+        <is>
+          <t>17-06-2027</t>
+        </is>
+      </c>
+      <c r="G53" s="18" t="inlineStr">
+        <is>
+          <t>CISO / Legal</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="inlineStr">
+        <is>
+          <t>Comité SGSI</t>
+        </is>
+      </c>
+      <c r="I53" s="20" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="J53" s="19" t="inlineStr">
+        <is>
+          <t>Interno</t>
+        </is>
+      </c>
+      <c r="K53" s="18" t="inlineStr">
+        <is>
+          <t>Cl. 4.2</t>
+        </is>
+      </c>
+      <c r="L53" s="18" t="inlineStr">
+        <is>
+          <t>Ley 21.663; Ley 19.628; PCI DSS v4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1" s="13">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>DOC-SGSI-03</t>
+        </is>
+      </c>
+      <c r="B54" s="18" t="inlineStr">
+        <is>
+          <t>Matriz de Competencias</t>
+        </is>
+      </c>
+      <c r="C54" s="19" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="D54" s="19" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E54" s="19" t="inlineStr">
+        <is>
+          <t>17-06-2026</t>
+        </is>
+      </c>
+      <c r="F54" s="19" t="inlineStr">
+        <is>
+          <t>17-06-2027</t>
+        </is>
+      </c>
+      <c r="G54" s="18" t="inlineStr">
+        <is>
+          <t>RRHH / CISO</t>
+        </is>
+      </c>
+      <c r="H54" s="18" t="inlineStr">
+        <is>
+          <t>Comité SGSI</t>
+        </is>
+      </c>
+      <c r="I54" s="20" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="J54" s="19" t="inlineStr">
+        <is>
+          <t>Interno</t>
+        </is>
+      </c>
+      <c r="K54" s="18" t="inlineStr">
+        <is>
+          <t>Cl. 7.2 · A.6.3</t>
+        </is>
+      </c>
+      <c r="L54" s="18" t="inlineStr">
+        <is>
+          <t>ISO 27001</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1" s="13">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>DOC-SGSI-04</t>
+        </is>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>Mapeo SGSI ↔ ISO 27001:2022 (Anexo A)</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E55" s="19" t="inlineStr">
+        <is>
+          <t>17-06-2026</t>
+        </is>
+      </c>
+      <c r="F55" s="19" t="inlineStr">
+        <is>
+          <t>17-06-2027</t>
+        </is>
+      </c>
+      <c r="G55" s="18" t="inlineStr">
+        <is>
+          <t>CISO</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr">
+        <is>
+          <t>CISO</t>
+        </is>
+      </c>
+      <c r="I55" s="20" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="J55" s="19" t="inlineStr">
+        <is>
+          <t>Interno</t>
+        </is>
+      </c>
+      <c r="K55" s="18" t="inlineStr">
+        <is>
+          <t>Anexo A</t>
+        </is>
+      </c>
+      <c r="L55" s="18" t="inlineStr">
+        <is>
+          <t>ISO 27001</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1" s="13">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>DOC-SGSI-05</t>
+        </is>
+      </c>
+      <c r="B56" s="18" t="inlineStr">
+        <is>
+          <t>Contrato de Trabajo y Anexo de Seguridad</t>
+        </is>
+      </c>
+      <c r="C56" s="19" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="D56" s="19" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E56" s="19" t="inlineStr">
+        <is>
+          <t>17-06-2026</t>
+        </is>
+      </c>
+      <c r="F56" s="19" t="inlineStr">
+        <is>
+          <t>17-06-2027</t>
+        </is>
+      </c>
+      <c r="G56" s="18" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="H56" s="18" t="inlineStr">
+        <is>
+          <t>Gerencia General</t>
+        </is>
+      </c>
+      <c r="I56" s="20" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="J56" s="19" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="K56" s="18" t="inlineStr">
+        <is>
+          <t>A.6.1, A.6.2, A.6.6</t>
+        </is>
+      </c>
+      <c r="L56" s="18" t="inlineStr">
+        <is>
+          <t>Ley 19.628; ISO Personas (6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1" s="13">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
           <t>EVI-SGSI-01</t>
         </is>
       </c>
-      <c r="B53" s="18" t="inlineStr">
+      <c r="B57" s="18" t="inlineStr">
         <is>
           <t>Repositorio de Evidencias del SGSI</t>
         </is>
       </c>
-      <c r="C53" s="19" t="inlineStr">
+      <c r="C57" s="19" t="inlineStr">
         <is>
           <t>Evidencias</t>
         </is>
       </c>
-      <c r="D53" s="19" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="E53" s="19" t="inlineStr">
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E57" s="19" t="inlineStr">
         <is>
           <t>17-06-2026</t>
         </is>
       </c>
-      <c r="F53" s="19" t="inlineStr">
+      <c r="F57" s="19" t="inlineStr">
         <is>
           <t>17-06-2027</t>
         </is>
       </c>
-      <c r="G53" s="18" t="inlineStr">
-        <is>
-          <t>CISO</t>
-        </is>
-      </c>
-      <c r="H53" s="18" t="inlineStr">
+      <c r="G57" s="18" t="inlineStr">
+        <is>
+          <t>CISO</t>
+        </is>
+      </c>
+      <c r="H57" s="18" t="inlineStr">
         <is>
           <t>Comité SGSI</t>
         </is>
       </c>
-      <c r="I53" s="20" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="J53" s="19" t="inlineStr">
-        <is>
-          <t>Interno</t>
-        </is>
-      </c>
-      <c r="K53" s="18" t="inlineStr">
+      <c r="I57" s="20" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="J57" s="19" t="inlineStr">
+        <is>
+          <t>Interno</t>
+        </is>
+      </c>
+      <c r="K57" s="18" t="inlineStr">
         <is>
           <t>Cl. 7.5, 9.1</t>
         </is>
       </c>
-      <c r="L53" s="18" t="inlineStr">
+      <c r="L57" s="18" t="inlineStr">
         <is>
           <t>NIST CSF GV.OV</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="21" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B54" s="22">
-        <f>COUNTA(A4:A53)</f>
+      <c r="B58" s="22">
+        <f>COUNTA(A4:A57)</f>
         <v/>
       </c>
-      <c r="C54" s="23" t="n"/>
-      <c r="D54" s="23" t="n"/>
-      <c r="E54" s="23" t="n"/>
-      <c r="F54" s="23" t="n"/>
-      <c r="G54" s="23" t="n"/>
-      <c r="H54" s="23" t="n"/>
-      <c r="I54" s="23" t="n"/>
-      <c r="J54" s="23" t="n"/>
-      <c r="K54" s="23" t="n"/>
-      <c r="L54" s="23" t="n"/>
+      <c r="C58" s="23" t="n"/>
+      <c r="D58" s="23" t="n"/>
+      <c r="E58" s="23" t="n"/>
+      <c r="F58" s="23" t="n"/>
+      <c r="G58" s="23" t="n"/>
+      <c r="H58" s="23" t="n"/>
+      <c r="I58" s="23" t="n"/>
+      <c r="J58" s="23" t="n"/>
+      <c r="K58" s="23" t="n"/>
+      <c r="L58" s="23" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:L53"/>
+  <autoFilter ref="A3:L57"/>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>

</xml_diff>

<commit_message>
Aplica retoques de revisión: enlaces clicables y matriz de competencias por organigrama
- Maestro Documental: nueva columna "Ubicación / Enlace" con link clicable a cada
  uno de los 54 documentos (URL de GitHub).
- Matriz Legal: nueva columna "Enlace a la ley (BCN)" con link directo a la norma;
  se suman Ley 21.459 (delitos informáticos), Ley 21.719 (datos personales),
  Código del Trabajo y Ley 19.496 (consumidor).
- Matriz de Competencias: roles reemplazados por el organigrama de NovaRetail
  (12 cargos: gerencia, finanzas, RRHH, ventas, compras, bodega, operaciones, TI),
  manteniendo las competencias de seguridad (O/D/—).
- READMEs (raíz y docs/) actualizados.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Maestro Documental SGSI.xlsx
+++ b/docs/Maestro Documental SGSI.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maestro Documental" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Maestro Documental'!$A$3:$L$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Maestro Documental'!$A$3:$M$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -99,8 +99,18 @@
       <color rgb="00006100"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -133,6 +143,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
   </fills>
@@ -170,7 +185,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -237,6 +252,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="12" min="1" max="1"/>
@@ -505,6 +526,7 @@
     <col width="13" customWidth="1" style="12" min="10" max="10"/>
     <col width="32" customWidth="1" style="12" min="11" max="11"/>
     <col width="28" customWidth="1" style="12" min="12" max="12"/>
+    <col width="34" customWidth="1" style="13" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="13">
@@ -582,6 +604,11 @@
           <t>Marcos relacionados</t>
         </is>
       </c>
+      <c r="M3" s="24" t="inlineStr">
+        <is>
+          <t>Ubicación / Enlace</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="28" customHeight="1" s="13">
       <c r="A4" s="17" t="inlineStr">
@@ -644,6 +671,11 @@
           <t>ISO 27001; NIST CSF GV.OC</t>
         </is>
       </c>
+      <c r="M4" s="25" t="inlineStr">
+        <is>
+          <t>Alcance del SGSI.md</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="28" customHeight="1" s="13">
       <c r="A5" s="17" t="inlineStr">
@@ -706,6 +738,11 @@
           <t>ISO 27001; PCI DSS; Ley 21.663; Ley 19.628</t>
         </is>
       </c>
+      <c r="M5" s="25" t="inlineStr">
+        <is>
+          <t>Politica General de Seguridad de la Informacion.md</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1" s="13">
       <c r="A6" s="17" t="inlineStr">
@@ -768,6 +805,11 @@
           <t>ISO 27001; NIST CSF GV.RR</t>
         </is>
       </c>
+      <c r="M6" s="25" t="inlineStr">
+        <is>
+          <t>Acta de Nombramiento CISO y Comite SGSI.md</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="28" customHeight="1" s="13">
       <c r="A7" s="17" t="inlineStr">
@@ -830,6 +872,11 @@
           <t>ISO 27001; NIST CSF GV.RR</t>
         </is>
       </c>
+      <c r="M7" s="25" t="inlineStr">
+        <is>
+          <t>Matriz RACI.md</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28" customHeight="1" s="13">
       <c r="A8" s="17" t="inlineStr">
@@ -892,6 +939,11 @@
           <t>ISO 27001; NIST CSF GV.OV</t>
         </is>
       </c>
+      <c r="M8" s="25" t="inlineStr">
+        <is>
+          <t>Procedimiento de Auditoria Interna.md</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1" s="13">
       <c r="A9" s="17" t="inlineStr">
@@ -954,6 +1006,11 @@
           <t>ISO 27001</t>
         </is>
       </c>
+      <c r="M9" s="25" t="inlineStr">
+        <is>
+          <t>Procedimiento de Revision por la Direccion.md</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1" s="13">
       <c r="A10" s="17" t="inlineStr">
@@ -1016,6 +1073,11 @@
           <t>ISO 27001; NIST CSF IMPROVE</t>
         </is>
       </c>
+      <c r="M10" s="25" t="inlineStr">
+        <is>
+          <t>Procedimiento de Gestion de No Conformidades y Acciones Correctivas.md</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="28" customHeight="1" s="13">
       <c r="A11" s="17" t="inlineStr">
@@ -1078,6 +1140,11 @@
           <t>ISO 27001; NIST CSF RECOVER</t>
         </is>
       </c>
+      <c r="M11" s="25" t="inlineStr">
+        <is>
+          <t>Plan de Continuidad del Negocio BCP-DRP.md</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1" s="13">
       <c r="A12" s="17" t="inlineStr">
@@ -1140,6 +1207,11 @@
           <t>ISO 27001</t>
         </is>
       </c>
+      <c r="M12" s="25" t="inlineStr">
+        <is>
+          <t>Objetivos de Seguridad de la Informacion.md</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="28" customHeight="1" s="13">
       <c r="A13" s="17" t="inlineStr">
@@ -1202,6 +1274,11 @@
           <t>PCI DSS Req 7, 8</t>
         </is>
       </c>
+      <c r="M13" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-01 - Política de control de acceso.docx</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="28" customHeight="1" s="13">
       <c r="A14" s="17" t="inlineStr">
@@ -1264,6 +1341,11 @@
           <t>PCI DSS Req 8</t>
         </is>
       </c>
+      <c r="M14" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-02 - Política de gestión de contraseñas y autenticación.docx</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="28" customHeight="1" s="13">
       <c r="A15" s="17" t="inlineStr">
@@ -1326,6 +1408,11 @@
           <t>PCI DSS Req 12.10</t>
         </is>
       </c>
+      <c r="M15" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-03 - Política de respaldo y recuperación.docx</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="28" customHeight="1" s="13">
       <c r="A16" s="17" t="inlineStr">
@@ -1388,6 +1475,11 @@
           <t>PCI DSS Req 5</t>
         </is>
       </c>
+      <c r="M16" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-04 - Política de protección contra malware.docx</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="28" customHeight="1" s="13">
       <c r="A17" s="17" t="inlineStr">
@@ -1450,6 +1542,11 @@
           <t>PCI DSS Req 6</t>
         </is>
       </c>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-05 - Política de gestión de parches y actualizacion.docx</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="28" customHeight="1" s="13">
       <c r="A18" s="17" t="inlineStr">
@@ -1512,6 +1609,11 @@
           <t>PCI DSS Req 1, 9</t>
         </is>
       </c>
+      <c r="M18" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-06 - Política de uso seguro de dispositivos y estac.docx</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="28" customHeight="1" s="13">
       <c r="A19" s="17" t="inlineStr">
@@ -1574,6 +1676,11 @@
           <t>PCI DSS Req 1, 4</t>
         </is>
       </c>
+      <c r="M19" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-07 - Política de seguridad de red.docx</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="28" customHeight="1" s="13">
       <c r="A20" s="17" t="inlineStr">
@@ -1636,6 +1743,11 @@
           <t>PCI DSS Req 10</t>
         </is>
       </c>
+      <c r="M20" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-08 - Política de registro y monitoreo.docx</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="28" customHeight="1" s="13">
       <c r="A21" s="17" t="inlineStr">
@@ -1698,6 +1810,11 @@
           <t>PCI DSS Req 6, 11</t>
         </is>
       </c>
+      <c r="M21" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-09 - Política de gestión de vulnerabilidades.docx</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="28" customHeight="1" s="13">
       <c r="A22" s="17" t="inlineStr">
@@ -1760,6 +1877,11 @@
           <t>Ley 19.628; PCI DSS Req 3, 9</t>
         </is>
       </c>
+      <c r="M22" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-10 - Política de manejo de información y clasificac.docx</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="28" customHeight="1" s="13">
       <c r="A23" s="17" t="inlineStr">
@@ -1822,6 +1944,11 @@
           <t>Ley 21.663; PCI DSS Req 12.10</t>
         </is>
       </c>
+      <c r="M23" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-11 - Política de gestión de incidentes y reporte ANCI.docx</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="28" customHeight="1" s="13">
       <c r="A24" s="17" t="inlineStr">
@@ -1884,6 +2011,11 @@
           <t>Ley 19.628; PCI DSS Req 3, 4</t>
         </is>
       </c>
+      <c r="M24" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-12 - Política de cifrado de datos.docx</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="28" customHeight="1" s="13">
       <c r="A25" s="17" t="inlineStr">
@@ -1946,6 +2078,11 @@
           <t>Ley 21.663; PCI DSS Req 12.8</t>
         </is>
       </c>
+      <c r="M25" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-13 - Política de gestión de proveedores y terceros OIV.docx</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="28" customHeight="1" s="13">
       <c r="A26" s="17" t="inlineStr">
@@ -2008,6 +2145,11 @@
           <t>Ley 19.628; ISO Personas (6)</t>
         </is>
       </c>
+      <c r="M26" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-14 - Política de contratación y desvinculación.docx</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="28" customHeight="1" s="13">
       <c r="A27" s="17" t="inlineStr">
@@ -2070,6 +2212,11 @@
           <t>PCI DSS Req 2, 6</t>
         </is>
       </c>
+      <c r="M27" s="25" t="inlineStr">
+        <is>
+          <t>POL-SGSI-15 - Política de línea base de software.docx</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="28" customHeight="1" s="13">
       <c r="A28" s="17" t="inlineStr">
@@ -2132,6 +2279,11 @@
           <t>PCI DSS Req 6</t>
         </is>
       </c>
+      <c r="M28" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-01 - Procedimiento de actualización y gestión de parches.docx</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="28" customHeight="1" s="13">
       <c r="A29" s="17" t="inlineStr">
@@ -2194,6 +2346,11 @@
           <t>PCI DSS Req 12.10</t>
         </is>
       </c>
+      <c r="M29" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-02 - Procedimiento de backup de base de datos.docx</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="28" customHeight="1" s="13">
       <c r="A30" s="17" t="inlineStr">
@@ -2256,6 +2413,11 @@
           <t>PCI DSS Req 6.5</t>
         </is>
       </c>
+      <c r="M30" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-03 - Procedimiento de rollback.docx</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="28" customHeight="1" s="13">
       <c r="A31" s="17" t="inlineStr">
@@ -2318,6 +2480,11 @@
           <t>PCI DSS Req 2, 6</t>
         </is>
       </c>
+      <c r="M31" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-04 - Procedimiento de línea base de software (Ansible).docx</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="28" customHeight="1" s="13">
       <c r="A32" s="17" t="inlineStr">
@@ -2380,6 +2547,11 @@
           <t>Ley 21.663; PCI DSS Req 12.10</t>
         </is>
       </c>
+      <c r="M32" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-05 - Procedimiento de incidentes con plazos ANCI.docx</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="28" customHeight="1" s="13">
       <c r="A33" s="17" t="inlineStr">
@@ -2442,6 +2614,11 @@
           <t>PCI DSS Req 7, 8</t>
         </is>
       </c>
+      <c r="M33" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-06 - Procedimiento de alta, modificación y baja de accesos.docx</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="28" customHeight="1" s="13">
       <c r="A34" s="17" t="inlineStr">
@@ -2504,6 +2681,11 @@
           <t>PCI DSS Req 7.2</t>
         </is>
       </c>
+      <c r="M34" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-07 - Procedimiento de revisión periódica de accesos.docx</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="28" customHeight="1" s="13">
       <c r="A35" s="17" t="inlineStr">
@@ -2566,6 +2748,11 @@
           <t>PCI DSS Req 8</t>
         </is>
       </c>
+      <c r="M35" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-08 - Procedimiento de uso del gestor de contraseñas.docx</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="28" customHeight="1" s="13">
       <c r="A36" s="17" t="inlineStr">
@@ -2628,6 +2815,11 @@
           <t>PCI DSS Req 1</t>
         </is>
       </c>
+      <c r="M36" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-09 - Procedimiento de segmentación y revisión de firewall.docx</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="28" customHeight="1" s="13">
       <c r="A37" s="17" t="inlineStr">
@@ -2690,6 +2882,11 @@
           <t>PCI DSS Req 10, 12.10</t>
         </is>
       </c>
+      <c r="M37" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-10 - Procedimiento de revisión y escalada de alertas.docx</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="28" customHeight="1" s="13">
       <c r="A38" s="17" t="inlineStr">
@@ -2752,6 +2949,11 @@
           <t>PCI DSS Req 11</t>
         </is>
       </c>
+      <c r="M38" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-11 - Procedimiento de escaneo de vulnerabilidades.docx</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="28" customHeight="1" s="13">
       <c r="A39" s="17" t="inlineStr">
@@ -2814,6 +3016,11 @@
           <t>Ley 19.628; PCI DSS Req 3.2</t>
         </is>
       </c>
+      <c r="M39" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-12 - Procedimiento de retención y eliminación segura.docx</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="28" customHeight="1" s="13">
       <c r="A40" s="17" t="inlineStr">
@@ -2876,6 +3083,11 @@
           <t>Ley 19.628; ISO Personas (6)</t>
         </is>
       </c>
+      <c r="M40" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-13 - Procedimiento de contratación y desvinculación.docx</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="28" customHeight="1" s="13">
       <c r="A41" s="17" t="inlineStr">
@@ -2938,6 +3150,11 @@
           <t>Ley 21.663; PCI DSS Req 12.8</t>
         </is>
       </c>
+      <c r="M41" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-14 - Procedimiento de evaluación de proveedores.docx</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="28" customHeight="1" s="13">
       <c r="A42" s="17" t="inlineStr">
@@ -3000,6 +3217,11 @@
           <t>PCI DSS Req 6</t>
         </is>
       </c>
+      <c r="M42" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-15 - Procedimiento de desarrollo seguro (SDLC).docx</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="28" customHeight="1" s="13">
       <c r="A43" s="17" t="inlineStr">
@@ -3062,6 +3284,11 @@
           <t>PCI DSS Req 5</t>
         </is>
       </c>
+      <c r="M43" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-16 - Procedimiento de respuesta ante malware.docx</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="28" customHeight="1" s="13">
       <c r="A44" s="17" t="inlineStr">
@@ -3124,6 +3351,11 @@
           <t>PCI DSS Req 9</t>
         </is>
       </c>
+      <c r="M44" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-17 - Procedimiento de uso seguro de dispositivos.docx</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="28" customHeight="1" s="13">
       <c r="A45" s="17" t="inlineStr">
@@ -3186,6 +3418,11 @@
           <t>Ley 19.628; PCI DSS Req 3, 4</t>
         </is>
       </c>
+      <c r="M45" s="25" t="inlineStr">
+        <is>
+          <t>PROC-SGSI-18 - Procedimiento de cifrado y gestión de llaves.docx</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="28" customHeight="1" s="13">
       <c r="A46" s="17" t="inlineStr">
@@ -3248,6 +3485,11 @@
           <t>ISO 27001; NIST CSF GV.RM/ID.RA</t>
         </is>
       </c>
+      <c r="M46" s="25" t="inlineStr">
+        <is>
+          <t>Metodologia de Evaluacion y Tratamiento de Riesgos.md</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="28" customHeight="1" s="13">
       <c r="A47" s="17" t="inlineStr">
@@ -3310,6 +3552,11 @@
           <t>ISO 27001; NIST CSF GV.RM</t>
         </is>
       </c>
+      <c r="M47" s="25" t="inlineStr">
+        <is>
+          <t>Plan de Tratamiento de Riesgos.md</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="28" customHeight="1" s="13">
       <c r="A48" s="17" t="inlineStr">
@@ -3372,6 +3619,11 @@
           <t>NIST CSF ID.AM</t>
         </is>
       </c>
+      <c r="M48" s="25" t="inlineStr">
+        <is>
+          <t>Analisis de Riesgos - Inventario, Matriz de Riesgos y SoA.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="28" customHeight="1" s="13">
       <c r="A49" s="17" t="inlineStr">
@@ -3434,6 +3686,11 @@
           <t>NIST CSF ID.RA</t>
         </is>
       </c>
+      <c r="M49" s="25" t="inlineStr">
+        <is>
+          <t>Analisis de Riesgos - Inventario, Matriz de Riesgos y SoA.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="28" customHeight="1" s="13">
       <c r="A50" s="17" t="inlineStr">
@@ -3496,6 +3753,11 @@
           <t>ISO 27001 Anexo A (cap. 8)</t>
         </is>
       </c>
+      <c r="M50" s="25" t="inlineStr">
+        <is>
+          <t>Analisis de Riesgos - Inventario, Matriz de Riesgos y SoA.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="28" customHeight="1" s="13">
       <c r="A51" s="17" t="inlineStr">
@@ -3558,6 +3820,11 @@
           <t>NIST CSF</t>
         </is>
       </c>
+      <c r="M51" s="25" t="inlineStr">
+        <is>
+          <t>Gap Analysis y Estado del SGSI.md</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="28" customHeight="1" s="13">
       <c r="A52" s="17" t="inlineStr">
@@ -3620,6 +3887,11 @@
           <t>ISO 27001</t>
         </is>
       </c>
+      <c r="M52" s="25" t="inlineStr">
+        <is>
+          <t>Maestro Documental SGSI.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="28" customHeight="1" s="13">
       <c r="A53" s="17" t="inlineStr">
@@ -3682,6 +3954,11 @@
           <t>Ley 21.663; Ley 19.628; PCI DSS v4.0</t>
         </is>
       </c>
+      <c r="M53" s="25" t="inlineStr">
+        <is>
+          <t>Matriz Legal.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="28" customHeight="1" s="13">
       <c r="A54" s="17" t="inlineStr">
@@ -3744,6 +4021,11 @@
           <t>ISO 27001</t>
         </is>
       </c>
+      <c r="M54" s="25" t="inlineStr">
+        <is>
+          <t>Matriz de Competencias.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="28" customHeight="1" s="13">
       <c r="A55" s="17" t="inlineStr">
@@ -3806,6 +4088,11 @@
           <t>ISO 27001</t>
         </is>
       </c>
+      <c r="M55" s="25" t="inlineStr">
+        <is>
+          <t>mapeo-iso27001.md</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="28" customHeight="1" s="13">
       <c r="A56" s="17" t="inlineStr">
@@ -3868,6 +4155,11 @@
           <t>Ley 19.628; ISO Personas (6)</t>
         </is>
       </c>
+      <c r="M56" s="25" t="inlineStr">
+        <is>
+          <t>Contrato de Trabajo y Anexo de Seguridad.docx</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="28" customHeight="1" s="13">
       <c r="A57" s="17" t="inlineStr">
@@ -3928,6 +4220,11 @@
       <c r="L57" s="18" t="inlineStr">
         <is>
           <t>NIST CSF GV.OV</t>
+        </is>
+      </c>
+      <c r="M57" s="25" t="inlineStr">
+        <is>
+          <t>README.md</t>
         </is>
       </c>
     </row>
@@ -3951,13 +4248,70 @@
       <c r="J58" s="23" t="n"/>
       <c r="K58" s="23" t="n"/>
       <c r="L58" s="23" t="n"/>
+      <c r="M58" s="23" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:L57"/>
+  <autoFilter ref="A3:M57"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId54"/>
+  </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Gobernanza: convierte los 9 documentos a .docx (Word) para SharePoint
- GOB-SGSI-01..09 pasan de .md a .docx (Word, generados con pandoc), listos para
  subir y vincular en SharePoint y consistentes con políticas y procedimientos.
- Elimina los .md de gobernanza (quedan en el historial de git); se conserva el
  README.md de la carpeta como índice.
- Actualiza enlaces a .docx en 00-gobernanza/README y en la columna
  "Ubicación / Enlace" del Maestro Documental.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Maestro Documental SGSI.xlsx
+++ b/docs/Maestro Documental SGSI.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="M4" s="25" t="inlineStr">
         <is>
-          <t>Alcance del SGSI.md</t>
+          <t>Alcance del SGSI.docx</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="M5" s="25" t="inlineStr">
         <is>
-          <t>Politica General de Seguridad de la Informacion.md</t>
+          <t>Politica General de Seguridad de la Informacion.docx</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="M6" s="25" t="inlineStr">
         <is>
-          <t>Acta de Nombramiento CISO y Comite SGSI.md</t>
+          <t>Acta de Nombramiento CISO y Comite SGSI.docx</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="M7" s="25" t="inlineStr">
         <is>
-          <t>Matriz RACI.md</t>
+          <t>Matriz RACI.docx</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="M8" s="25" t="inlineStr">
         <is>
-          <t>Procedimiento de Auditoria Interna.md</t>
+          <t>Procedimiento de Auditoria Interna.docx</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="M9" s="25" t="inlineStr">
         <is>
-          <t>Procedimiento de Revision por la Direccion.md</t>
+          <t>Procedimiento de Revision por la Direccion.docx</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="M10" s="25" t="inlineStr">
         <is>
-          <t>Procedimiento de Gestion de No Conformidades y Acciones Correctivas.md</t>
+          <t>Procedimiento de Gestion de No Conformidades y Acciones Correctivas.docx</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="M11" s="25" t="inlineStr">
         <is>
-          <t>Plan de Continuidad del Negocio BCP-DRP.md</t>
+          <t>Plan de Continuidad del Negocio BCP-DRP.docx</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="M12" s="25" t="inlineStr">
         <is>
-          <t>Objetivos de Seguridad de la Informacion.md</t>
+          <t>Objetivos de Seguridad de la Informacion.docx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Análisis: convierte los 3 documentos a .docx (Word) para SharePoint
- Metodología de Evaluación y Tratamiento de Riesgos (ANR-01), Plan de Tratamiento
  de Riesgos (ANR-02) y Gap Analysis pasan de .md a .docx (pandoc), listos para
  subir y vincular en SharePoint.
- Elimina los .md (quedan en el historial); se conserva README.md como índice.
- Actualiza enlaces a .docx en 04-analisis/README y en el Maestro Documental.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Maestro Documental SGSI.xlsx
+++ b/docs/Maestro Documental SGSI.xlsx
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M46" s="25" t="inlineStr">
         <is>
-          <t>Metodologia de Evaluacion y Tratamiento de Riesgos.md</t>
+          <t>Metodologia de Evaluacion y Tratamiento de Riesgos.docx</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="M47" s="25" t="inlineStr">
         <is>
-          <t>Plan de Tratamiento de Riesgos.md</t>
+          <t>Plan de Tratamiento de Riesgos.docx</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="M51" s="25" t="inlineStr">
         <is>
-          <t>Gap Analysis y Estado del SGSI.md</t>
+          <t>Gap Analysis y Estado del SGSI.docx</t>
         </is>
       </c>
     </row>

</xml_diff>